<commit_message>
refactor: aplicar POM estricto y agregar Playwright Fixtures
- Mover selectores directos de step-definitions a Page Objects (LoginPage,
  RegisterPage): fillCredentials(), isAccountPageVisible(),
  isAccountDropdownVisible(), submitBtn getter, errorAlertLocator getter
- Reemplazar expect().toBeVisible() dentro de Page Objects por
  .waitFor({ state: 'visible' }) — las assertions pertenecen a los steps,
  no a los Page Objects (regla POM del documento academico)
- Eliminar import de expect/@playwright/test en Page Objects que no hacen
  assertions; usan solo 'playwright' para selectores y acciones
- Crear src/fixtures/base.fixture.ts con Playwright Fixtures para todos
  los Page Objects y una pagina pre-autenticada (requisito de arquitectura)
- Todos los step-definitions delegan 100% de selectores a Page Objects

Resultado: 6 scenarios (6 passed) / 42 steps (42 passed)
</commit_message>
<xml_diff>
--- a/test-data/datos_prueba.xlsx
+++ b/test-data/datos_prueba.xlsx
@@ -116,10 +116,10 @@
     <t>110111</t>
   </si>
   <si>
-    <t>30814</t>
-  </si>
-  <si>
-    <t>2026-06-02T16:57:20.109Z</t>
+    <t>30820</t>
+  </si>
+  <si>
+    <t>2026-06-03T01:56:58.494Z</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
chore: actualizar dependencias y datos de prueba
- @types/node actualizado a 22.19.19
- package-lock.json sincronizado
- datos_prueba.xlsx con resultados de la ultima ejecucion (numero_confirmacion y fecha_activacion)
</commit_message>
<xml_diff>
--- a/test-data/datos_prueba.xlsx
+++ b/test-data/datos_prueba.xlsx
@@ -116,10 +116,10 @@
     <t>110111</t>
   </si>
   <si>
-    <t>30820</t>
-  </si>
-  <si>
-    <t>2026-06-03T01:56:58.494Z</t>
+    <t>30829</t>
+  </si>
+  <si>
+    <t>2026-06-04T15:45:04.566Z</t>
   </si>
 </sst>
 </file>

</xml_diff>